<commit_message>
Fixed bugs in data; exported CSV files
</commit_message>
<xml_diff>
--- a/InputData/bldgs/SYDEC/Start Year Distributed Electricity Capacity.xlsx
+++ b/InputData/bldgs/SYDEC/Start Year Distributed Electricity Capacity.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10211"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ssy02/Desktop/Brazil/eps-us-3.4.2/InputData/bldgs/SYDEC/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saido\Documents\eps-brazil-cpl\InputData\bldgs\SYDEC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{309FE6C2-FA0D-094C-BC74-60C106784ED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="21380" tabRatio="670" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="765" windowWidth="34200" windowHeight="21375" tabRatio="670" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -42,7 +41,7 @@
     <definedName name="Table5_A">'[1]AEO21 Table 5'!$A$29:$A$58</definedName>
     <definedName name="Table5_A_22">'[1]AEO22 Table 5'!$A$29:$A$58</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -233,7 +232,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
@@ -430,7 +429,7 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -447,24 +446,25 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="16">
-    <cellStyle name="Body: normal cell" xfId="5" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
-    <cellStyle name="Body: normal cell 2" xfId="11" xr:uid="{716C4B1B-8246-4F86-B207-AA505C13595A}"/>
-    <cellStyle name="Font: Calibri, 9pt regular" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
-    <cellStyle name="Footnotes: top row" xfId="6" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
-    <cellStyle name="Footnotes: top row 2" xfId="10" xr:uid="{C2ED02E1-753F-4A0F-8FE2-481788A509A5}"/>
-    <cellStyle name="Header: bottom row" xfId="2" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
-    <cellStyle name="Header: bottom row 2" xfId="13" xr:uid="{F75A30F3-6D8D-40F3-86A8-B4BC9C0FBFE4}"/>
-    <cellStyle name="Header: top rows" xfId="9" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
-    <cellStyle name="Hyperlink" xfId="15" builtinId="8"/>
+    <cellStyle name="Body: normal cell" xfId="5"/>
+    <cellStyle name="Body: normal cell 2" xfId="11"/>
+    <cellStyle name="Font: Calibri, 9pt regular" xfId="1"/>
+    <cellStyle name="Footnotes: top row" xfId="6"/>
+    <cellStyle name="Footnotes: top row 2" xfId="10"/>
+    <cellStyle name="Header: bottom row" xfId="2"/>
+    <cellStyle name="Header: bottom row 2" xfId="13"/>
+    <cellStyle name="Header: top rows" xfId="9"/>
+    <cellStyle name="Lien hypertexte" xfId="15" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="7" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
-    <cellStyle name="Parent row" xfId="4" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
-    <cellStyle name="Parent row 2" xfId="12" xr:uid="{8C867030-DF57-4EB8-AF9D-C18BC478B3D2}"/>
-    <cellStyle name="Percent" xfId="8" builtinId="5"/>
-    <cellStyle name="Table title" xfId="3" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
-    <cellStyle name="Table title 2" xfId="14" xr:uid="{49152C00-9ED6-45AE-B892-720EA6B7E8AB}"/>
+    <cellStyle name="Normal 2" xfId="7"/>
+    <cellStyle name="Parent row" xfId="4"/>
+    <cellStyle name="Parent row 2" xfId="12"/>
+    <cellStyle name="Pourcentage" xfId="8" builtinId="5"/>
+    <cellStyle name="Table title" xfId="3"/>
+    <cellStyle name="Table title 2" xfId="14"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -499,7 +499,7 @@
         <xdr:cNvPr id="2" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{52E8FB2A-AD19-4574-B8DD-F27040DF5DA4}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{52E8FB2A-AD19-4574-B8DD-F27040DF5DA4}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -549,7 +549,7 @@
         <xdr:cNvPr id="3" name="Picture 10">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{46CA9E6F-FF7B-4CD0-B424-9280B1CA04E7}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{46CA9E6F-FF7B-4CD0-B424-9280B1CA04E7}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -604,7 +604,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{69C2E308-D0C8-4344-8780-93A610808AC8}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{69C2E308-D0C8-4344-8780-93A610808AC8}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -634,7 +634,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="About"/>
@@ -12837,7 +12837,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="About"/>
@@ -12868,9 +12868,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -12908,9 +12908,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -12945,7 +12945,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -12980,7 +12980,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -13153,19 +13153,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B46"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="51" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
@@ -13173,122 +13173,122 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B5" s="2">
         <v>2017</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B8" s="5" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B12" s="2">
         <v>2017</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B15" s="5" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B22" s="3" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B24" s="2">
         <v>2017</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B27" s="5" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>9</v>
       </c>
@@ -13296,76 +13296,76 @@
         <v>52</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B33" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="1"/>
       <c r="B37" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="4"/>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="4"/>
       <c r="B39" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B42" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>56</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B8" r:id="rId1" xr:uid="{12ED9C53-7F03-4991-94D4-39F7D1819083}"/>
-    <hyperlink ref="B15" r:id="rId2" xr:uid="{95745DF3-A1DA-4CB7-99D9-0C2BA0FC1C29}"/>
-    <hyperlink ref="B27" r:id="rId3" xr:uid="{A0BBEDE5-488D-400D-93C3-5CE202925DCB}"/>
+    <hyperlink ref="B8" r:id="rId1"/>
+    <hyperlink ref="B15" r:id="rId2"/>
+    <hyperlink ref="B27" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId4"/>
@@ -13373,39 +13373,39 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E12ABA5A-AE0D-4838-9DAF-2D52F3C51B9A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AL34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>0.2</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>28</v>
       </c>
@@ -13413,7 +13413,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>30</v>
       </c>
@@ -13421,7 +13421,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>31</v>
       </c>
@@ -13429,7 +13429,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="31" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
         <v>24</v>
       </c>
@@ -13542,7 +13542,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="32" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:38" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
         <v>33</v>
       </c>
@@ -13655,7 +13655,7 @@
         <v>37000</v>
       </c>
     </row>
-    <row r="33" spans="2:38" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:38" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
         <v>34</v>
       </c>
@@ -13768,7 +13768,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="34" spans="2:38" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:38" x14ac:dyDescent="0.25">
       <c r="D34" s="9"/>
     </row>
   </sheetData>
@@ -13778,49 +13778,49 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2C6E203-4B87-471D-ADB1-18059C3FD476}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:AL21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>0.2</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="19" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:38" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>40</v>
       </c>
@@ -13933,7 +13933,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="20" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:38" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>41</v>
       </c>
@@ -14046,7 +14046,7 @@
         <v>6.78</v>
       </c>
     </row>
-    <row r="21" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:38" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
         <v>42</v>
       </c>
@@ -14166,17 +14166,17 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="4" width="23.5" customWidth="1"/>
+    <col min="1" max="4" width="23.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>19</v>
       </c>
@@ -14190,7 +14190,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -14204,7 +14204,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -14218,7 +14218,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -14232,7 +14232,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -14246,7 +14246,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -14262,23 +14262,24 @@
         <v>700</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>3</v>
       </c>
       <c r="B7" s="11">
-        <f>('Solar PV'!G21*10^6)*(1-'Solar PV'!$A$8)</f>
-        <v>532800</v>
+        <f>('Solar PV'!G21*10^3)*(1-'Solar PV'!$A$8)</f>
+        <v>532.80000000000007</v>
       </c>
       <c r="C7" s="11">
         <v>0</v>
       </c>
       <c r="D7" s="11">
-        <f>('Solar PV'!I21*10^6)*'Solar PV'!$A$8</f>
-        <v>192000.00000000003</v>
-      </c>
+        <f>('Solar PV'!I21*10^3)*'Solar PV'!$A$8</f>
+        <v>192.00000000000003</v>
+      </c>
+      <c r="F7" s="12"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -14292,7 +14293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -14306,7 +14307,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>6</v>
       </c>
@@ -14320,7 +14321,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>7</v>
       </c>
@@ -14334,7 +14335,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -14348,7 +14349,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -14362,7 +14363,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>15</v>
       </c>
@@ -14376,7 +14377,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>16</v>
       </c>
@@ -14390,7 +14391,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>17</v>
       </c>
@@ -14404,7 +14405,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>18</v>
       </c>

</xml_diff>